<commit_message>
Update noise tools and add textured 3D orbit visualization
</commit_message>
<xml_diff>
--- a/noise/gradiometer_noise_calculator_updated_2.xlsx
+++ b/noise/gradiometer_noise_calculator_updated_2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lindeman\OneDrive - JPL\Documents\Python\gradiometer\noise\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jpl365prod-my.sharepoint.com/personal/mark_a_lindeman_jpl_nasa_gov/Documents/Documents/Python/gradiometer/noise/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122D72A0-86E5-4E00-9B3E-5487FF2143D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="11_0D0151F95AF7142B87B02F66859576EBEA21AC47" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8CA64E3-EB78-4253-9DA2-230A7D2A2AFB}"/>
   <bookViews>
-    <workbookView xWindow="39450" yWindow="-3465" windowWidth="38700" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28665" yWindow="-30" windowWidth="38700" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="53">
   <si>
     <t>Gradiometer Noise Calculator</t>
   </si>
@@ -41,6 +41,9 @@
     <t>Inputs</t>
   </si>
   <si>
+    <t>10 m gradiometer, SQUID</t>
+  </si>
+  <si>
     <t>Coefficient lookup (from central-difference stencils)</t>
   </si>
   <si>
@@ -119,7 +122,16 @@
     <t>Characteristic frequency f_char [Hz] where ASD(f_char)*sqrt(BW)=required sensor RMS</t>
   </si>
   <si>
-    <t>1/f ASD coefficient at 1 Hz from SQUID model [fT/sqrt(Hz)]</t>
+    <t>Sensor</t>
+  </si>
+  <si>
+    <t>HTS SQUID</t>
+  </si>
+  <si>
+    <t>Fluxgate</t>
+  </si>
+  <si>
+    <t>1/f ASD coefficient at 1 Hz from sensor model [fT/sqrt(Hz)]</t>
   </si>
   <si>
     <t>Integrated 1/f sensor RMS over band [pT]</t>
@@ -128,12 +140,24 @@
     <t>Trial frequency for 1/f ASD [Hz]</t>
   </si>
   <si>
+    <t>reference for noise</t>
+  </si>
+  <si>
+    <t>Cantor et al IEEE TRANSACTIONSON APPLIED SUPERCONDUCTIVITY, VOL. 5, NO. 2, JUNE 1995</t>
+  </si>
+  <si>
+    <t>Kivelson  Space Science Reviews (2023) 219:48</t>
+  </si>
+  <si>
     <t>1/f sensor ASD at trial frequency [pT/sqrt(Hz)]</t>
   </si>
   <si>
     <t>1/f sensor ASD at trial frequency [fT/sqrt(Hz)]</t>
   </si>
   <si>
+    <t>Margin factor</t>
+  </si>
+  <si>
     <t>Notes:</t>
   </si>
   <si>
@@ -152,10 +176,22 @@
     <t>- Integrated 1/f RMS over [f_low, f_high]: RMS = (A_1Hz/1000)*SQRT(LN(f_high/f_low)) [pT].</t>
   </si>
   <si>
-    <t>Margin factor</t>
-  </si>
-  <si>
-    <t>Maximum allowed 2/f noise at trial freq   [pT/sqrt(Hz)]</t>
+    <t>Maximum allowed 1/f noise at trial freq   [pT/sqrt(Hz)]</t>
+  </si>
+  <si>
+    <t>1 m gradiometer, SQUID</t>
+  </si>
+  <si>
+    <t>10 cm gradiometer, SQUID</t>
+  </si>
+  <si>
+    <t>10 m gradiometer, flux gatee</t>
+  </si>
+  <si>
+    <t>100 km gradiometer flux gate</t>
+  </si>
+  <si>
+    <t>100 m gradiometer flux gate</t>
   </si>
 </sst>
 </file>
@@ -169,7 +205,7 @@
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -206,6 +242,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -296,7 +340,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -324,9 +368,14 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="168" fontId="5" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -349,16 +398,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>590550</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
+      <xdr:col>23</xdr:col>
       <xdr:colOff>38580</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>55638</xdr:rowOff>
+      <xdr:rowOff>59448</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -682,428 +731,1062 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="80.6640625" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="5" max="5" width="18.109375" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="2" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="21.5546875" customWidth="1"/>
+    <col min="7" max="7" width="25.44140625" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
       <c r="D1" s="27"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="B3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2">
         <v>10</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E4" s="2">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2">
+        <v>100000</v>
+      </c>
+      <c r="G4" s="2">
+        <v>1000</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="J4" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="2">
         <v>2</v>
       </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C5" s="2">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2</v>
+      </c>
+      <c r="E5" s="2">
+        <v>2</v>
+      </c>
+      <c r="F5" s="2">
+        <v>2</v>
+      </c>
+      <c r="G5" s="2">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6">
         <v>2</v>
       </c>
-      <c r="F6">
+      <c r="J6">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" s="18">
         <v>1</v>
       </c>
-      <c r="E7">
+      <c r="C7" s="18">
+        <v>1</v>
+      </c>
+      <c r="D7" s="18">
+        <v>1</v>
+      </c>
+      <c r="E7" s="18">
+        <v>1</v>
+      </c>
+      <c r="F7" s="18">
+        <v>1</v>
+      </c>
+      <c r="G7" s="18">
+        <v>1</v>
+      </c>
+      <c r="I7">
         <v>3</v>
       </c>
-      <c r="F7">
+      <c r="J7">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3">
         <f>1/3600</f>
         <v>2.7777777777777778E-4</v>
       </c>
-      <c r="E8">
+      <c r="C8" s="3">
+        <f>1/3600</f>
+        <v>2.7777777777777778E-4</v>
+      </c>
+      <c r="D8" s="3">
+        <f>1/3600</f>
+        <v>2.7777777777777778E-4</v>
+      </c>
+      <c r="E8" s="3">
+        <f>1/3600</f>
+        <v>2.7777777777777778E-4</v>
+      </c>
+      <c r="F8" s="3">
+        <f>1/3600</f>
+        <v>2.7777777777777778E-4</v>
+      </c>
+      <c r="G8" s="3">
+        <f>1/3600</f>
+        <v>2.7777777777777778E-4</v>
+      </c>
+      <c r="I8">
         <v>5</v>
       </c>
-      <c r="F8">
+      <c r="J8">
         <v>14.444444444444439</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" s="3">
         <f>1/114.483</f>
         <v>8.7349213420333145E-3</v>
       </c>
-      <c r="E9">
+      <c r="C9" s="3">
+        <f>1/114.483</f>
+        <v>8.7349213420333145E-3</v>
+      </c>
+      <c r="D9" s="3">
+        <f>1/114.483</f>
+        <v>8.7349213420333145E-3</v>
+      </c>
+      <c r="E9" s="3">
+        <f>1/114.483</f>
+        <v>8.7349213420333145E-3</v>
+      </c>
+      <c r="F9" s="3">
+        <f>1/114.483</f>
+        <v>8.7349213420333145E-3</v>
+      </c>
+      <c r="G9" s="3">
+        <f>1/114.483</f>
+        <v>8.7349213420333145E-3</v>
+      </c>
+      <c r="I9">
         <v>7</v>
       </c>
-      <c r="F9">
+      <c r="J9">
         <v>42.139999999999993</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I10">
         <v>9</v>
       </c>
-      <c r="F10">
+      <c r="J10">
         <v>87.227392290249398</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11">
+        <v>13</v>
+      </c>
+      <c r="I11">
         <v>11</v>
       </c>
-      <c r="F11">
+      <c r="J11">
         <v>150.95518392542391</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" s="10">
-        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(B5,$E$5:$E$29,$F$5:$F$29)),NA())</f>
+        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(B5,$I$5:$I$29,$J$5:$J$29)),NA())</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C12" s="10">
+        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(C5,$I$5:$I$29,$J$5:$J$29)),NA())</f>
+        <v>2</v>
+      </c>
+      <c r="D12" s="10">
+        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(D5,$I$5:$I$29,$J$5:$J$29)),NA())</f>
+        <v>2</v>
+      </c>
+      <c r="E12" s="10">
+        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(E5,$I$5:$I$29,$J$5:$J$29)),NA())</f>
+        <v>2</v>
+      </c>
+      <c r="F12" s="10">
+        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(F5,$I$5:$I$29,$J$5:$J$29)),NA())</f>
+        <v>2</v>
+      </c>
+      <c r="G12" s="10">
+        <f>IFERROR(_xlfn.SINGLE(_xlfn.XLOOKUP(G5,$I$5:$I$29,$J$5:$J$29)),NA())</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13" s="5">
         <f>IF(B6="gradient",B12/(B4^2),B12)</f>
         <v>0.02</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C13" s="5">
+        <f>IF(C6="gradient",C12/(C4^2),C12)</f>
+        <v>2</v>
+      </c>
+      <c r="D13" s="5">
+        <f>IF(D6="gradient",D12/(D4^2),D12)</f>
+        <v>199.99999999999997</v>
+      </c>
+      <c r="E13" s="5">
+        <f>IF(E6="gradient",E12/(E4^2),E12)</f>
+        <v>0.02</v>
+      </c>
+      <c r="F13" s="5">
+        <f>IF(F6="gradient",F12/(F4^2),F12)</f>
+        <v>2.0000000000000001E-10</v>
+      </c>
+      <c r="G13" s="5">
+        <f>IF(G6="gradient",G12/(G4^2),G12)</f>
+        <v>1.9999999999999999E-6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14" s="12">
         <f>B7/SQRT(B13)</f>
         <v>7.0710678118654755</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C14" s="12">
+        <f>C7/SQRT(C13)</f>
+        <v>0.70710678118654746</v>
+      </c>
+      <c r="D14" s="12">
+        <f>D7/SQRT(D13)</f>
+        <v>7.0710678118654766E-2</v>
+      </c>
+      <c r="E14" s="12">
+        <f>E7/SQRT(E13)</f>
+        <v>7.0710678118654755</v>
+      </c>
+      <c r="F14" s="12">
+        <f>F7/SQRT(F13)</f>
+        <v>70710.678118654745</v>
+      </c>
+      <c r="G14" s="12">
+        <f>G7/SQRT(G13)</f>
+        <v>707.10678118654755</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B15" s="5">
         <f>B9-B8</f>
         <v>8.4571435642555367E-3</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C15" s="5">
+        <f>C9-C8</f>
+        <v>8.4571435642555367E-3</v>
+      </c>
+      <c r="D15" s="5">
+        <f>D9-D8</f>
+        <v>8.4571435642555367E-3</v>
+      </c>
+      <c r="E15" s="5">
+        <f>E9-E8</f>
+        <v>8.4571435642555367E-3</v>
+      </c>
+      <c r="F15" s="5">
+        <f>F9-F8</f>
+        <v>8.4571435642555367E-3</v>
+      </c>
+      <c r="G15" s="5">
+        <f>G9-G8</f>
+        <v>8.4571435642555367E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16" s="11">
         <f>B14/SQRT(B15)</f>
         <v>76.890582439195114</v>
       </c>
-      <c r="E16" t="s">
-        <v>18</v>
-      </c>
-      <c r="F16">
+      <c r="C16" s="11">
+        <f>C14/SQRT(C15)</f>
+        <v>7.6890582439195105</v>
+      </c>
+      <c r="D16" s="11">
+        <f>D14/SQRT(D15)</f>
+        <v>0.76890582439195132</v>
+      </c>
+      <c r="E16" s="11">
+        <f>E14/SQRT(E15)</f>
+        <v>76.890582439195114</v>
+      </c>
+      <c r="F16" s="11">
+        <f>F14/SQRT(F15)</f>
+        <v>768905.82439195109</v>
+      </c>
+      <c r="G16" s="11">
+        <f>G14/SQRT(G15)</f>
+        <v>7689.0582439195114</v>
+      </c>
+      <c r="I16" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16">
         <f>B16*SQRT($B$15)</f>
         <v>7.0710678118654755</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B17" s="11"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B18" s="6"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B19" s="6"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B20" s="11">
         <f>B14^2/LN(B9/B8)</f>
         <v>14.500054993115885</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C20" s="11">
+        <f>C14^2/LN(C9/C8)</f>
+        <v>0.1450005499311588</v>
+      </c>
+      <c r="D20" s="11">
+        <f>D14^2/LN(D9/D8)</f>
+        <v>1.4500054993115889E-3</v>
+      </c>
+      <c r="E20" s="11">
+        <f>E14^2/LN(E9/E8)</f>
+        <v>14.500054993115885</v>
+      </c>
+      <c r="F20" s="11">
+        <f>F14^2/LN(F9/F8)</f>
+        <v>1450005499.311588</v>
+      </c>
+      <c r="G20" s="11">
+        <f>G14^2/LN(G9/G8)</f>
+        <v>145000.54993115886</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B21" s="11"/>
-    </row>
-    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+    </row>
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B22" s="9">
         <f>SQRT(B20/((B8+B9)/2))</f>
         <v>56.724723300480704</v>
       </c>
-      <c r="E22" t="s">
-        <v>18</v>
-      </c>
-      <c r="F22">
+      <c r="C22" s="9">
+        <f>SQRT(C20/((C8+C9)/2))</f>
+        <v>5.6724723300480697</v>
+      </c>
+      <c r="D22" s="9">
+        <f>SQRT(D20/((D8+D9)/2))</f>
+        <v>0.56724723300480717</v>
+      </c>
+      <c r="E22" s="9">
+        <f>SQRT(E20/((E8+E9)/2))</f>
+        <v>56.724723300480704</v>
+      </c>
+      <c r="F22" s="9">
+        <f>SQRT(F20/((F8+F9)/2))</f>
+        <v>567247.23300480691</v>
+      </c>
+      <c r="G22" s="9">
+        <f>SQRT(G20/((G8+G9)/2))</f>
+        <v>5672.4723300480709</v>
+      </c>
+      <c r="I22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J22">
         <f>B22*SQRT($B$15)</f>
         <v>5.2165603685496462</v>
       </c>
-      <c r="H22" t="s">
-        <v>22</v>
-      </c>
-      <c r="I22">
-        <f>F22/$B$14</f>
+      <c r="L22" t="s">
+        <v>23</v>
+      </c>
+      <c r="M22">
+        <f>J22/$B$14</f>
         <v>0.73773304221409008</v>
       </c>
     </row>
-    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B23" s="13">
         <f>(B8+B9)/2</f>
         <v>4.5063495599055462E-3</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="C23" s="13">
+        <f>(C8+C9)/2</f>
+        <v>4.5063495599055462E-3</v>
+      </c>
+      <c r="D23" s="13">
+        <f>(D8+D9)/2</f>
+        <v>4.5063495599055462E-3</v>
+      </c>
+      <c r="E23" s="13">
+        <f>(E8+E9)/2</f>
+        <v>4.5063495599055462E-3</v>
+      </c>
+      <c r="F23" s="13">
+        <f>(F8+F9)/2</f>
+        <v>4.5063495599055462E-3</v>
+      </c>
+      <c r="G23" s="13">
+        <f>(G8+G9)/2</f>
+        <v>4.5063495599055462E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="B24" s="9"/>
-    </row>
-    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+    </row>
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B25" s="8">
         <f>SQRT(B20/SQRT(B8*B9))</f>
         <v>96.481867315635242</v>
       </c>
-      <c r="E25" t="s">
-        <v>18</v>
-      </c>
-      <c r="F25">
+      <c r="C25" s="8">
+        <f>SQRT(C20/SQRT(C8*C9))</f>
+        <v>9.6481867315635217</v>
+      </c>
+      <c r="D25" s="8">
+        <f>SQRT(D20/SQRT(D8*D9))</f>
+        <v>0.96481867315635261</v>
+      </c>
+      <c r="E25" s="8">
+        <f>SQRT(E20/SQRT(E8*E9))</f>
+        <v>96.481867315635242</v>
+      </c>
+      <c r="F25" s="8">
+        <f>SQRT(F20/SQRT(F8*F9))</f>
+        <v>964818.67315635236</v>
+      </c>
+      <c r="G25" s="8">
+        <f>SQRT(G20/SQRT(G8*G9))</f>
+        <v>9648.1867315635245</v>
+      </c>
+      <c r="I25" t="s">
+        <v>19</v>
+      </c>
+      <c r="J25">
         <f>B25*SQRT($B$15)</f>
         <v>8.8727358378871646</v>
       </c>
-      <c r="H25" t="s">
-        <v>22</v>
-      </c>
-      <c r="I25">
-        <f>F25/$B$14</f>
+      <c r="L25" t="s">
+        <v>23</v>
+      </c>
+      <c r="M25">
+        <f>J25/$B$14</f>
         <v>1.2547943357293836</v>
       </c>
     </row>
-    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B26" s="13">
         <f>SQRT(B8*B9)</f>
         <v>1.5576800183136775E-3</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C26" s="13">
+        <f>SQRT(C8*C9)</f>
+        <v>1.5576800183136775E-3</v>
+      </c>
+      <c r="D26" s="13">
+        <f>SQRT(D8*D9)</f>
+        <v>1.5576800183136775E-3</v>
+      </c>
+      <c r="E26" s="13">
+        <f>SQRT(E8*E9)</f>
+        <v>1.5576800183136775E-3</v>
+      </c>
+      <c r="F26" s="13">
+        <f>SQRT(F8*F9)</f>
+        <v>1.5576800183136775E-3</v>
+      </c>
+      <c r="G26" s="13">
+        <f>SQRT(G8*G9)</f>
+        <v>1.5576800183136775E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="7"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" s="15">
         <f>SQRT(B20/B29)</f>
         <v>76.890582439195114</v>
       </c>
-      <c r="E28" t="s">
-        <v>18</v>
-      </c>
-      <c r="F28">
+      <c r="C28" s="15">
+        <f>SQRT(C20/C29)</f>
+        <v>7.6890582439195105</v>
+      </c>
+      <c r="D28" s="15">
+        <f>SQRT(D20/D29)</f>
+        <v>0.76890582439195121</v>
+      </c>
+      <c r="E28" s="15">
+        <f>SQRT(E20/E29)</f>
+        <v>76.890582439195114</v>
+      </c>
+      <c r="F28" s="15">
+        <f>SQRT(F20/F29)</f>
+        <v>768905.82439195109</v>
+      </c>
+      <c r="G28" s="15">
+        <f>SQRT(G20/G29)</f>
+        <v>7689.0582439195114</v>
+      </c>
+      <c r="I28" t="s">
+        <v>19</v>
+      </c>
+      <c r="J28">
         <f>B28*SQRT($B$15)</f>
         <v>7.0710678118654755</v>
       </c>
-      <c r="H28" t="s">
-        <v>22</v>
-      </c>
-      <c r="I28">
-        <f>F28/$B$14</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L28" t="s">
+        <v>23</v>
+      </c>
+      <c r="M28">
+        <f>J28/$B$14</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" s="17">
         <f>B20*B15/(B14^2)</f>
         <v>2.4525809353276272E-3</v>
       </c>
-      <c r="E29" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C29" s="17">
+        <f>C20*C15/(C14^2)</f>
+        <v>2.4525809353276268E-3</v>
+      </c>
+      <c r="D29" s="17">
+        <f>D20*D15/(D14^2)</f>
+        <v>2.4525809353276272E-3</v>
+      </c>
+      <c r="E29" s="17">
+        <f>E20*E15/(E14^2)</f>
+        <v>2.4525809353276272E-3</v>
+      </c>
+      <c r="F29" s="17">
+        <f>F20*F15/(F14^2)</f>
+        <v>2.4525809353276272E-3</v>
+      </c>
+      <c r="G29" s="17">
+        <f>G20*G15/(G14^2)</f>
+        <v>2.4525809353276272E-3</v>
+      </c>
+      <c r="I29" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B30" s="8"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>28</v>
-      </c>
-      <c r="B31" s="20">
+        <v>29</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" s="20">
         <v>22.5167</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>29</v>
-      </c>
-      <c r="B32" s="24">
-        <f>SQRT((B31/1000)^2*LN(B9/B8))</f>
+      <c r="C32" s="20">
+        <v>22.5167</v>
+      </c>
+      <c r="D32" s="20">
+        <v>22.5167</v>
+      </c>
+      <c r="E32" s="20">
+        <f>1000*E37*SQRT(E35)</f>
+        <v>100000</v>
+      </c>
+      <c r="F32" s="20">
+        <f>1000*F37*SQRT(F35)</f>
+        <v>100000</v>
+      </c>
+      <c r="G32" s="20">
+        <f>1000*G37*SQRT(G35)</f>
+        <v>100000</v>
+      </c>
+      <c r="J32" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" s="24">
+        <f>SQRT((B32/1000)^2*LN(B9/B8))</f>
         <v>4.1812382921966061E-2</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="23"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>30</v>
-      </c>
-      <c r="B34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C33" s="24">
+        <f>SQRT((C32/1000)^2*LN(C9/C8))</f>
+        <v>4.1812382921966061E-2</v>
+      </c>
+      <c r="D33" s="24">
+        <f>SQRT((D32/1000)^2*LN(D9/D8))</f>
+        <v>4.1812382921966061E-2</v>
+      </c>
+      <c r="E33" s="25">
+        <f>SQRT((E32/1000)^2*LN(E9/E8))</f>
+        <v>185.69498604132067</v>
+      </c>
+      <c r="F33" s="25">
+        <f>SQRT((F32/1000)^2*LN(F9/F8))</f>
+        <v>185.69498604132067</v>
+      </c>
+      <c r="G33" s="25">
+        <f>SQRT((G32/1000)^2*LN(G9/G8))</f>
+        <v>185.69498604132067</v>
+      </c>
+      <c r="J33" s="20">
+        <v>22.5167</v>
+      </c>
+      <c r="K33" s="20">
+        <f>1000*K38*SQRT(K36)</f>
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="J34" s="24">
+        <f>SQRT((J33/1000)^2*LN(J10/J9))</f>
+        <v>1.9205583659552449E-2</v>
+      </c>
+      <c r="K34" s="25" t="e">
+        <f>SQRT((K33/1000)^2*LN(K10/K9))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>31</v>
-      </c>
-      <c r="B35" s="21">
-        <f>(B31/1000)/SQRT(B34)</f>
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
+        <v>1</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="J35" s="23"/>
+      <c r="K35" s="23"/>
+    </row>
+    <row r="36" spans="1:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J36">
+        <v>1</v>
+      </c>
+      <c r="K36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="21">
+        <f>(B32/1000)/SQRT(B35)</f>
         <v>2.2516700000000001E-2</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>32</v>
-      </c>
-      <c r="B36" s="20">
-        <f>1000*B35</f>
+      <c r="C37" s="21">
+        <f>(C32/1000)/SQRT(C35)</f>
+        <v>2.2516700000000001E-2</v>
+      </c>
+      <c r="D37" s="21">
+        <f>(D32/1000)/SQRT(D35)</f>
+        <v>2.2516700000000001E-2</v>
+      </c>
+      <c r="E37" s="21">
+        <v>100</v>
+      </c>
+      <c r="F37" s="21">
+        <v>100</v>
+      </c>
+      <c r="G37" s="21">
+        <v>100</v>
+      </c>
+      <c r="J37" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="K37" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38" s="20">
+        <f>1000*B37</f>
         <v>22.5167</v>
       </c>
-      <c r="C36" s="20"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B38" s="22">
-        <f>B14/B32</f>
+      <c r="C38" s="20">
+        <f>1000*C37</f>
+        <v>22.5167</v>
+      </c>
+      <c r="D38" s="20">
+        <f>1000*D37</f>
+        <v>22.5167</v>
+      </c>
+      <c r="E38" s="20">
+        <f>1000*E37</f>
+        <v>100000</v>
+      </c>
+      <c r="F38" s="20">
+        <f>1000*F37</f>
+        <v>100000</v>
+      </c>
+      <c r="G38" s="20">
+        <f>1000*G37</f>
+        <v>100000</v>
+      </c>
+      <c r="J38" s="21">
+        <f>(J33/1000)/SQRT(J36)</f>
+        <v>2.2516700000000001E-2</v>
+      </c>
+      <c r="K38" s="21">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="20"/>
+      <c r="J39" s="20">
+        <f>1000*J38</f>
+        <v>22.5167</v>
+      </c>
+      <c r="K39" s="20">
+        <f>1000*K38</f>
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" s="22">
+        <f>B14/B33</f>
         <v>169.11420296379958</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B39" s="25">
-        <f>B35*B38</f>
+      <c r="C40" s="30">
+        <f>C14/C33</f>
+        <v>16.911420296379955</v>
+      </c>
+      <c r="D40" s="30">
+        <f>D14/D33</f>
+        <v>1.691142029637996</v>
+      </c>
+      <c r="E40" s="29">
+        <f>E14/E33</f>
+        <v>3.8078937738749867E-2</v>
+      </c>
+      <c r="F40" s="22">
+        <f>F14/F33</f>
+        <v>380.78937738749863</v>
+      </c>
+      <c r="G40" s="28">
+        <f>G14/G33</f>
+        <v>3.8078937738749867</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" s="31">
+        <f>B37*B40</f>
         <v>3.8078937738749863</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C41" s="32">
+        <f>C37*C40</f>
+        <v>0.38078937738749852</v>
+      </c>
+      <c r="D41" s="32">
+        <f>D37*D40</f>
+        <v>3.8078937738749867E-2</v>
+      </c>
+      <c r="E41" s="31">
+        <f>E37*E40</f>
+        <v>3.8078937738749867</v>
+      </c>
+      <c r="F41" s="31">
+        <f>F37*F40</f>
+        <v>38078.937738749861</v>
+      </c>
+      <c r="G41" s="31">
+        <f>G37*G40</f>
+        <v>380.78937738749869</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="4"/>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="4"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="4"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>

</xml_diff>